<commit_message>
feat: fix fan capacity white highlight, add Yoon XP mod, clean up artist dropdown
- Add .skill-white CSS class to properly render white border on fan capacity skills
- Add 240/DPS Attacking Group Center and 10% Gain Fans to white/violet highlights
- Remove header row "Arist" from artist dropdown by requiring numeric mod value
- Alphabetize artist XP modifier dropdown
- Add Yoon to artistxpmods.xlsx (0% extra cost, Community Event)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/artistxpmods.xlsx
+++ b/src/artistxpmods.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mick/Documents/ApexGirl/apexgirl/src/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mick/Documents/ApexGirl/kts-unified/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{938FC745-8775-904B-BC99-834AAF1600E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40878817-1138-054E-A3A2-FAF84BF78663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="2700" windowWidth="27640" windowHeight="16940" xr2:uid="{180760AF-A946-4C4D-894E-EC2D1266BA43}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="102">
   <si>
     <t>INCREASED EXP COST PER GIRL</t>
   </si>
@@ -339,6 +339,9 @@
   </si>
   <si>
     <t>Arist</t>
+  </si>
+  <si>
+    <t>Yoon</t>
   </si>
 </sst>
 </file>
@@ -749,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A65215-58F0-4641-94E3-D836F01989B2}">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1131,41 +1134,41 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>41</v>
+        <v>101</v>
       </c>
       <c r="B28" s="4">
         <v>0</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B29" s="4">
         <v>0</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B30" s="4">
         <v>0</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>44</v>
@@ -1173,13 +1176,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B31" s="4">
         <v>0</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>44</v>
@@ -1187,13 +1190,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B32" s="4">
         <v>0</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>44</v>
@@ -1201,7 +1204,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B33" s="4">
         <v>0</v>
@@ -1215,13 +1218,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B34" s="4">
         <v>0</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>44</v>
@@ -1229,13 +1232,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B35" s="4">
         <v>0</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>44</v>
@@ -1243,13 +1246,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B36" s="4">
         <v>0</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>44</v>
@@ -1257,13 +1260,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B37" s="4">
         <v>0</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>44</v>
@@ -1271,13 +1274,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B38" s="4">
         <v>0</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>44</v>
@@ -1285,7 +1288,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B39" s="4">
         <v>0</v>
@@ -1299,13 +1302,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40" s="4">
         <v>0</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>44</v>
@@ -1313,13 +1316,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B41" s="4">
         <v>0</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>44</v>
@@ -1327,13 +1330,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B42" s="4">
         <v>0</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>44</v>
@@ -1341,13 +1344,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B43" s="4">
         <v>0</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>44</v>
@@ -1355,13 +1358,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B44" s="4">
         <v>0</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>44</v>
@@ -1369,27 +1372,27 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B45" s="4">
         <v>0</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B46" s="4">
         <v>0</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>62</v>
@@ -1397,13 +1400,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B47" s="4">
         <v>0</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>62</v>
@@ -1411,13 +1414,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B48" s="4">
         <v>0</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>62</v>
@@ -1425,13 +1428,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B49" s="4">
         <v>0</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>62</v>
@@ -1439,27 +1442,27 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B50" s="4">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B51" s="4">
         <v>0.2</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>68</v>
@@ -1467,13 +1470,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B52" s="4">
         <v>0.2</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>68</v>
@@ -1481,27 +1484,27 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B53" s="4">
         <v>0.2</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B54" s="4">
         <v>0.2</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>72</v>
@@ -1509,13 +1512,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B55" s="4">
         <v>0.2</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>72</v>
@@ -1523,27 +1526,27 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B56" s="4">
-        <v>0.44</v>
+        <v>0.2</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B57" s="4">
         <v>0.44</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>76</v>
@@ -1551,13 +1554,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B58" s="4">
         <v>0.44</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>76</v>
@@ -1565,27 +1568,27 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B59" s="4">
-        <v>0</v>
+        <v>0.44</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B60" s="4">
         <v>0</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>80</v>
@@ -1593,27 +1596,27 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B61" s="4">
         <v>0</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B62" s="4">
         <v>0</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>83</v>
@@ -1621,13 +1624,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B63" s="4">
         <v>0</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>83</v>
@@ -1635,13 +1638,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B64" s="4">
         <v>0</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>83</v>
@@ -1649,13 +1652,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B65" s="4">
         <v>0</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>83</v>
@@ -1663,27 +1666,27 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B66" s="4">
         <v>0</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B67" s="4">
         <v>0</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>89</v>
@@ -1691,13 +1694,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B68" s="4">
         <v>0</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>89</v>
@@ -1705,27 +1708,27 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B69" s="4">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B70" s="4">
         <v>0.2</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>93</v>
@@ -1733,13 +1736,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B71" s="4">
         <v>0.2</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>93</v>
@@ -1747,27 +1750,27 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B72" s="4">
-        <v>0.44</v>
+        <v>0.2</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B73" s="4">
         <v>0.44</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>97</v>
@@ -1775,15 +1778,29 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B74" s="4">
         <v>0.44</v>
       </c>
       <c r="C74" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B75" s="4">
+        <v>0.44</v>
+      </c>
+      <c r="C75" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D74" s="3" t="s">
+      <c r="D75" s="3" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>